<commit_message>
Match protein substitution name forms in supplement search
</commit_message>
<xml_diff>
--- a/tests/fixtures/article/supplements/28944238-axin2-st2.xlsx
+++ b/tests/fixtures/article/supplements/28944238-axin2-st2.xlsx
@@ -2392,7 +2392,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>F0000X</t>
+          <t>p.Pro245Serfs</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -2412,7 +2412,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>P245S</t>
+          <t>p.Pro245Ser</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -2432,7 +2432,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>F0000X</t>
+          <t>P245S1</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">

</xml_diff>